<commit_message>
Excluir Cátedra USP y Citibeats (decisión del equipo); mantener los 3 borde
Tras el análisis profundo y la discusión con el criterio inclusivo del equipo:
- BR Cátedra/Co:Lab USP -> NO: investigación en curso sin despliegue con
  ciudadanos ni proceso propio (crítico: estudio sin despliegue).
- CO Citibeats+PNUD -> NO: escucha social de redes sin proceso convocado
  (crítico: misma regla que U-Report).
- Se MANTIENEN con nota: BR Brasil Participativo clustering (producción no
  confirmada; reevaluar 2027), BR OPA Piauí (validar IA con SEPLAN) y BR São
  Paulo Gemini (análisis complementario, patrón Pol.is/LUC).

Set final: 33 SÍ · 32 iniciativas efectivas · 74 NO. Prom regional 2026 = 25
(2025 misma metodología = 25, Δ 0; BR 80, CO 63). Docs de frontera y análisis
profundo actualizados; todas las planillas regeneradas.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/calculo_indice_2025vs2026_ILIA2026.xlsx
+++ b/data/gates/calculo_indice_2025vs2026_ILIA2026.xlsx
@@ -542,16 +542,16 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -593,13 +593,13 @@
         <v>66</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -860,10 +860,10 @@
       <c r="C16" s="3" t="inlineStr"/>
       <c r="D16" s="3" t="inlineStr"/>
       <c r="E16" s="5" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17">
@@ -876,7 +876,7 @@
       <c r="C17" s="3" t="inlineStr"/>
       <c r="D17" s="3" t="inlineStr"/>
       <c r="E17" s="5" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F17" s="3" t="inlineStr"/>
     </row>
@@ -939,57 +939,57 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>82</v>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>+7</t>
-        </is>
+        <v>63</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>-19</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>4</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>78</v>
-      </c>
-      <c r="E3" s="7" t="n">
-        <v>-4</v>
+        <v>80</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>+5</t>
+        </is>
       </c>
       <c r="F3" s="3" t="n">
         <v>4</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -1373,18 +1373,16 @@
         <v>25</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>28</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19">
@@ -1398,10 +1396,10 @@
         <v>46</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="F19" s="3" t="inlineStr"/>
       <c r="G19" s="3" t="inlineStr"/>
@@ -1537,16 +1535,16 @@
         <v>100</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>75</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>0</v>
@@ -1582,7 +1580,7 @@
         <v>66</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>2</v>
@@ -1998,7 +1996,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>34 iniciativas efectivas: clasificación final SÍ (tras validación manual), respetando el dedup.</t>
+          <t>32 iniciativas efectivas: clasificación final SÍ (tras validación manual), respetando el dedup.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planilla de cálculo: comparación en 3 columnas (2025 antigua · 2025 nueva · 2026)
La pestaña 2 ahora muestra: 2025 con la metodología 2025 (recalculado con el
motor legacy validado desde la BBDD, desviación máx. 1 pt vs el oficial
publicado), 2025 con la metodología nueva y 2026 con la metodología nueva.
Se agregan dos deltas que descomponen el cambio: Δ metodología (misma base
2025, fórmula nueva vs antigua) y Δ datos (misma fórmula, base 2026 vs 2025).
Nota de lectura al pie y supuestos actualizados.

Regional: 26 (met. antigua) -> 25 (met. nueva, efecto metodología -1) -> 25
(datos 2026, efecto datos 0).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/calculo_indice_2025vs2026_ILIA2026.xlsx
+++ b/data/gates/calculo_indice_2025vs2026_ILIA2026.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="1 · Índice 2026" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2 · 2025 vs 2026 (misma met.)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2 · 2025 ant · 2025 nva · 2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="3 · Sub-Uso 2026 (detalle)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="4 · Supuestos y método" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +34,11 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00777777"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -94,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -118,6 +123,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -891,19 +899,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>País</t>
@@ -912,25 +922,40 @@
       <c r="B1" s="1" t="inlineStr"/>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Indicador 2025</t>
+          <t>2025
+met. 2025 (oficial)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Indicador 2026</t>
+          <t>2025
+met. nueva</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Δ (2026−2025)</t>
+          <t>2026
+met. nueva</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Δ metodología
+(2025 nva − 2025 ant)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Δ datos
+(2026 − 2025 nva)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Nº inic. 2025</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Nº inic. 2026</t>
         </is>
@@ -948,20 +973,26 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
+        <v>76</v>
+      </c>
+      <c r="D2" s="3" t="n">
         <v>75</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="E2" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>+15</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="H2" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="I2" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -977,18 +1008,24 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
+        <v>84</v>
+      </c>
+      <c r="D3" s="3" t="n">
         <v>82</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="E3" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="E3" s="7" t="n">
+      <c r="F3" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G3" s="7" t="n">
         <v>-22</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="H3" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="I3" s="3" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1004,20 +1041,26 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="D4" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="E4" s="3" t="n">
         <v>74</v>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="7" t="n">
+        <v>-7</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>+24</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="H4" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="I4" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1033,127 +1076,161 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="D5" s="3" t="n">
         <v>46</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="E5" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="F5" s="7" t="n">
+        <v>-8</v>
+      </c>
+      <c r="G5" s="7" t="n">
         <v>-22</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="H5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="I5" s="3" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Costa Rica</t>
+          <t>México</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>-44</v>
-      </c>
-      <c r="F6" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>-12</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="3" t="n">
-        <v>0</v>
+      <c r="I6" s="3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HN</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Honduras</t>
+          <t>Costa Rica</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>-9</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>1</v>
+        <v>44</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>-44</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>HN</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Honduras</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>-8</v>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>-9</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="3" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="D9" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="D9" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>-2</v>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>2</v>
+      <c r="E9" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>-8</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1171,17 +1248,23 @@
         <v>0</v>
       </c>
       <c r="D10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="F10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>+34</t>
         </is>
       </c>
-      <c r="F10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="3" t="n">
+      <c r="H10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1197,18 +1280,26 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D11" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="D11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="n">
         <v>-32</v>
       </c>
-      <c r="F11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="3" t="n">
+      <c r="H11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1224,18 +1315,26 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D12" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="E12" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="n">
         <v>-5</v>
       </c>
-      <c r="F12" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="3" t="n">
+      <c r="H12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1251,18 +1350,26 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="D13" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="E13" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="n">
         <v>-4</v>
       </c>
-      <c r="F13" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="3" t="n">
+      <c r="H13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1281,17 +1388,23 @@
         <v>0</v>
       </c>
       <c r="D14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="F14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>+25</t>
         </is>
       </c>
-      <c r="F14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="3" t="n">
+      <c r="H14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1310,17 +1423,23 @@
         <v>0</v>
       </c>
       <c r="D15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="F15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>+23</t>
         </is>
       </c>
-      <c r="F15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="3" t="n">
+      <c r="H15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1339,17 +1458,23 @@
         <v>0</v>
       </c>
       <c r="D16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="F16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>+20</t>
         </is>
       </c>
-      <c r="F16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="3" t="n">
+      <c r="H16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1361,6 +1486,8 @@
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr"/>
@@ -1370,41 +1497,39 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>25</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="G18" s="3" t="n">
+      <c r="I18" s="3" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Promedio (países con iniciativas)</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>46</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>38</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>-8</v>
-      </c>
-      <c r="F19" s="3" t="inlineStr"/>
-      <c r="G19" s="3" t="inlineStr"/>
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Lectura: 'Δ metodología' aísla el efecto del cambio de fórmula sobre la MISMA base 2025; 'Δ datos' aísla el efecto del cambio de base (salidas+nuevas) con la MISMA fórmula nueva. Columna '2025 met. 2025': recalculado con el motor legacy desde la BBDD (desviación máx. vs oficial publicado = 1 pt).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B19:I19"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1957,7 +2082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1965,96 +2090,108 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>CÁLCULO DEL ÍNDICE — 2026 preliminar y comparación 2025 vs 2026</t>
         </is>
       </c>
-      <c r="B1" s="9" t="n"/>
+      <c r="B1" s="10" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr"/>
-      <c r="B2" s="9" t="inlineStr"/>
+      <c r="A2" s="11" t="inlineStr"/>
+      <c r="B2" s="10" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Qué es</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Cálculo preliminar y determinístico con los datos actuales. La comparación usa la MISMA metodología (CENIA v2) sobre ambas bases, para aislar el efecto del cambio de datos (no de fórmula).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Set 2026</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>33 iniciativas efectivas: clasificación final SÍ (tras validación manual), respetando el dedup.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Set 2025</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>28 iniciativas del baseline 2025 (como estaban en el índice 2025), recodificadas a la taxonomía 2026 y corridas con la metodología nueva.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2025 metodología antigua</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Columna adicional en la pestaña 2: recalculado con el motor legacy desde la BBDD (desviación máx. vs oficial publicado = 1 pt). Junto a las otras dos permite separar el EFECTO METODOLOGÍA (misma base 2025, fórmula nueva vs antigua) del EFECTO DATOS (misma fórmula nueva, base 2026 vs 2025).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Metodología</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>CENIA v2 (jun-2026). Indicador = (Sub-Uso + Sub-Desarrollo)/2. Sub-Uso = promedio de 5: Tipos de proceso (÷5) · Etapas (÷4) · Continuidad = nivel máx. del país (÷3) · Organización Convocante (3 sub-componentes: gub ÷3 + no-gub ÷4 + co-convocatoria por máx. relativo) · Cantidad = todas las elegibles (umbrales 0/25/50/75/100). Sub-Desarrollo = 2025 (desarrollador nac/int × 4 tipos, máx. relativo + tipos de IA).</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Redondeo</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>legacy · count_min_level=0 · escenario=A</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Nota máx. relativo</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>El Sub-Desarrollo y la co-convocatoria usan máximo relativo POR CICLO: cada base (2025 y 2026) se normaliza contra su propio máximo, como indica la metodología.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Aviso</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Preliminar. Es una foto con los datos de hoy; los valores pueden cambiar si se completan gaps o se ajustan casos frontera.</t>
         </is>

</xml_diff>